<commit_message>
CD1 exploration adding fat/bw and lean/bw as well as modifications in length and grid
</commit_message>
<xml_diff>
--- a/data/echoMRI/Kotz04012026.xlsx
+++ b/data/echoMRI/Kotz04012026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr backupFile="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carosandovalcab/Documents/GitHub/data/data/echoMRI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carosandovalcaballero/Documents/GitHub/data/data/echoMRI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5ED8A3C-54FA-5145-A356-0AB438BBB728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFD0F95-1CEB-B24F-B1E4-98FC70F08463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="44800" windowHeight="25200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtractedScans" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>RecNumber</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t>9452</t>
-  </si>
-  <si>
-    <t>9554</t>
   </si>
   <si>
     <t>9455</t>
@@ -551,7 +548,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -580,7 +577,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -609,7 +606,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -638,7 +635,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -667,7 +664,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -696,7 +693,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -725,7 +722,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -738,8 +735,8 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
+      <c r="B9">
+        <v>9454</v>
       </c>
       <c r="C9">
         <v>15.71</v>
@@ -754,7 +751,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -768,7 +765,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10">
         <v>13.46</v>
@@ -783,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -797,7 +794,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11">
         <v>8.3699999999999992</v>
@@ -812,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -826,7 +823,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12">
         <v>6.76</v>
@@ -841,7 +838,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -855,7 +852,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13">
         <v>8.25</v>
@@ -870,7 +867,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -884,7 +881,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14">
         <v>8.5</v>
@@ -899,7 +896,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -913,7 +910,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -928,7 +925,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -942,7 +939,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C16">
         <v>4.34</v>
@@ -957,7 +954,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -971,7 +968,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17">
         <v>6.81</v>
@@ -986,7 +983,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1000,7 +997,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18">
         <v>1.35</v>
@@ -1015,7 +1012,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H18">
         <v>1</v>

</xml_diff>